<commit_message>
Completed GenAI scope and AP pillar workflow and evaluation
</commit_message>
<xml_diff>
--- a/Publications/GenAI/1_prompt_debugging/Dave_borderline/borderline.xlsx
+++ b/Publications/GenAI/1_prompt_debugging/Dave_borderline/borderline.xlsx
@@ -624,6 +624,23 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
 </styleSheet>
 </file>
 
@@ -804,7 +821,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I1048576"/>
   <sheetFormatPr defaultColWidth="8.34375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="10" min="1" style="1" width="8.34"/>
@@ -912,7 +929,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="3276.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>26</v>
       </c>
@@ -1673,6 +1690,7 @@
         <v>34</v>
       </c>
     </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="B2:C2"/>

</xml_diff>